<commit_message>
feat: Context Fabric P4 dual-write, Story Codex, writer-friendly stylometry
- P4: dual-write 8 junctions → references (relationships, factions, wields,
  location/idea connections, chapter cast, power combos, location entities)
- Story Codex (/codex): navigable wiki built from references graph
- Stylometry deepening UI: pacing heatmap (C3), Burrows Δ (#3), rolling drift
  (#4), voice distance (C2) + plain-language verdict layer, tiered disclosure,
  metric tooltips, actionable hints
- docs: prune done/blocked plans (consistency-guardian removed)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-cases.xlsx
+++ b/test-cases.xlsx
@@ -14,6 +14,8 @@
     <sheet name="UX ที่แก้" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Quick Wins" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Stylometry เจาะลึก" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Context Fabric P4" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Story Codex (B1)" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ผู้ช่วย AI (ใหม่)'!$A$1:$G$19</definedName>
@@ -21,7 +23,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'บรรณารักษ์ + กราฟ'!$A$1:$G$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'UX ที่แก้'!$A$1:$G$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Quick Wins'!$A$1:$G$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Stylometry เจาะลึก'!$A$1:$G$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Stylometry เจาะลึก'!$A$1:$G$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Context Fabric P4'!$A$1:$G$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Story Codex (B1)'!$A$1:$G$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -507,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -670,6 +674,26 @@
       </c>
       <c r="B16" t="n">
         <v>13</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Context Fabric P4</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Story Codex (B1)</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -2757,7 +2781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3183,8 +3207,971 @@
       <c r="F14" s="6" t="inlineStr"/>
       <c r="G14" s="6" t="inlineStr"/>
     </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>WF-01</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>[สรุปคน] กล่องสรุปบนสุด</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>เลือกตอนในแดชบอร์ดวิเคราะห์สไตล์</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>เห็นกล่องสรุปภาษาคน (headline + bullet) อยู่"บนสุด"ของการ์ด ก่อนตัวเลข/กราฟ</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr"/>
+      <c r="G15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>WF-02</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>[สรุปคน] ตอนต่างจากเล่มมาก</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>เลือกตอนที่ maxZ ≥ 1.96</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>headline "ตอนนี้ต่างจากเล่มชัดเจน" (เหลือง) + note "ถ้าตั้งใจ (flashback/เปลี่ยนมุมมอง/ไคลแม็กซ์) ไม่ต้องกังวล"</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr"/>
+      <c r="G16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>WF-03</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>[สรุปคน] ตอนกลมกลืน</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>เลือกตอนที่ทุกมิติ |z|&lt;1</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>headline "กลมกลืนกับทั้งเล่ม" (เขียว) + "ทุกมิติอยู่ในช่วงปกติของคุณ"</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr"/>
+      <c r="G17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>WF-04</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>[สรุปคน] bullet แปลถูกทิศ</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>ตอนที่ burstiness สูง / บทสนทนาเยอะ</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>bullet เป็นภาษาคน เช่น "จังหวะ: สั้น-ยาวสลับแรง", "บทสนทนา: บทสนทนาเยอะ" (z&gt;0=high, z&lt;0=low)</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr"/>
+      <c r="G18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>WF-05</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>[tiered] ตัวเลขดิบพับ default</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>เปิดการ์ดตอน</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>grid z-score รายมิติ "ถูกซ่อน" → มีปุ่ม "ดูตัวเลขเชิงลึก (z-score รายมิติ)" กดแล้วค่อยเห็น</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr"/>
+      <c r="G19" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G14"/>
+  <autoFilter ref="A1:G19"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>หัวข้อ</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>เงื่อนไข / ขั้นตอน</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>ผลที่คาดหวัง</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>ความสำคัญ</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>ผลทดสอบ</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>หมายเหตุ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>CF-01</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>ความสัมพันธ์ตัวละคร → กราฟ</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>สร้างความสัมพันธ์ A↔B (หน้า Relationships/Characters) → เปิด World Graph</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>เห็นเส้นเชื่อม A–B (related_to) ในกราฟ</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr"/>
+      <c r="G2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>CF-02</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>ลบความสัมพันธ์ → เส้นหาย</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>ลบความสัมพันธ์ A↔B → รีเฟรช World Graph</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>เส้น related_to A–B หายไป</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr"/>
+      <c r="G3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>CF-03</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>สมาชิกก๊ก → กราฟ</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>เพิ่มตัวละครเข้าก๊ก (member) → World Graph</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>เห็นเส้น character→faction (member_of)</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>CF-04</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>ออกจากก๊ก → เส้นหาย</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>ลบสมาชิกออกจากก๊ก</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>เส้น member_of หายจากกราฟ</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>CF-05</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>assign พลัง → กราฟ</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>มอบพลังให้ตัวละคร (power manager)</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>เห็นเส้น character→power (wields)</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr"/>
+      <c r="G6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>CF-06</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>ถอนพลัง → เส้นหาย</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>ลบพลังจากตัวละคร</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>เส้น wields หายจากกราฟ</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>CF-07</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>เชื่อมสถานที่ → กราฟ</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>สร้าง location connection</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>เห็นเส้น location→location (connects_to)</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr"/>
+      <c r="G8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>CF-08</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>เชื่อมไอเดีย → กราฟ</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>สร้าง idea connection แบบ related (และแบบ ancestor)</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>related → linked_to, ancestor → derived_from ปรากฏในกราฟ</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr"/>
+      <c r="G9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>CF-09</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>สูตรผสมพลัง → กราฟ</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>สร้าง power combination (ต้นทาง 2 พลัง → ผลลัพธ์)</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>เห็นเส้น combines_into จากทุกพลังต้นทาง → พลังผลลัพธ์</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr"/>
+      <c r="G10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>CF-10</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>ตัวละครในบท → กราฟ</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>เพิ่มตัวละครเข้าบท (chapter cast)</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>เห็นเส้น chapter→character (features) — หมายเหตุ: chapter ถูกซ่อน default ในกราฟ เปิดที่ legend ก่อน</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr"/>
+      <c r="G11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>CF-11</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>สิ่งมีชีวิตในสถานที่ → กราฟ</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>assign entity (สัตว์/สิ่งมีชีวิต) เข้า location</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>เห็นเส้น entity→location (inhabits)</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>ต่ำ</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr"/>
+      <c r="G12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>CF-12</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Librarian เห็นเชื่อมโยงครบขึ้น</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>หลังเชื่อม member_of/wields แล้ว ถามบรรณารักษ์ "X สังกัดก๊กไหน / มีพลังอะไร"</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>ตอบได้จากความเชื่อมโยงที่เพิ่ง dual-write (ต้อง Vector Sync ถ้าใช้ vector)</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr"/>
+      <c r="G13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>CF-13</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>ของเดิมไม่พัง</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>เพิ่ม/ลบ junction ต่างๆ ผ่าน UI ปกติ</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>ทุกอย่างทำงานเหมือนเดิม (dual-write เป็น additive ไม่กระทบ flow เดิม)</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr"/>
+      <c r="G14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>CF-14</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>ไม่มี edge ซ้ำ</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>เชื่อมความสัมพันธ์เดิมซ้ำ (ถ้า UI ยอม) หรือแก้ค่า</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>references ไม่มี edge ซ้ำ (addReference เป็น upsert บน from+to+relation)</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>ต่ำ</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr"/>
+      <c r="G15" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G15"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>หัวข้อ</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>เงื่อนไข / ขั้นตอน</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>ผลที่คาดหวัง</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>ความสำคัญ</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>ผลทดสอบ</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>หมายเหตุ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>SC-01</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>เปิดหน้า Story Codex</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>sidebar กลุ่ม "สร้างโลก" &gt; Story Codex</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>เห็นรายการ entity ทางซ้าย จัดกลุ่มตามชนิด (ตัวละคร/สถานที่/พลัง/ก๊ก...) พร้อมจำนวน</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr"/>
+      <c r="G2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>SC-02</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>ค้นหาในคลัง</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>พิมพ์ในช่องค้นหา</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>รายการกรองตามชื่อ (เฉพาะที่ตรง)</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr"/>
+      <c r="G3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>SC-03</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>เลือก entity → ความเชื่อมโยง</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>คลิกตัวละคร/สถานที่ใดๆ</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>ฝั่งขวาแสดงชื่อ + ชนิด + ส่วน "เชื่อมโยงไป" / "ถูกอ้างถึงโดย" ตาม references</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>SC-04</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>navigate ในคลัง</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>คลิกความเชื่อมโยงในฝั่งขวา</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>กระโดดไปดู entity ปลายทางใน codex (เดินสำรวจต่อได้)</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>SC-05</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>เปิดหน้าเต็ม</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>กด "เปิดหน้าเต็ม" ของ entity</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>ไปหน้าจริงของ entity (เช่น /characters/[id]) ตาม href</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr"/>
+      <c r="G6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>SC-06</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>entity ไม่มีความเชื่อมโยง</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>เลือก entity ที่ยังไม่ได้เชื่อมอะไร</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>แสดง "ยังไม่มีความเชื่อมโยง — ลองเชื่อมในหน้า..."</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>ต่ำ</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>SC-07</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>นิยายว่าง</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>นิยายที่ยังไม่มี entity/reference</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>empty state "ยังไม่มีข้อมูลในคลังเรื่อง"</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>ต่ำ</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr"/>
+      <c r="G8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>SC-08</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>ป้าย relation ไทย</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>ดูความเชื่อมโยงหลายแบบ</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>แสดงเป็นไทย: สังกัด / ครอบครองพลัง / สัมพันธ์กับ / เชื่อมไป / อาศัยที่ ฯลฯ</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>ต่ำ</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr"/>
+      <c r="G9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>SC-09</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>สะท้อน P4 ทันที</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>เชื่อม member_of หรือ wields ในหน้าอื่น แล้วกลับมา codex (รีเฟรช)</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>ความเชื่อมโยงใหม่ปรากฏ (reuse getNovelGraph อ่านจาก references ที่ P4 dual-write)</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr"/>
+      <c r="G10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>SC-10</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>chapter/note แสดงด้วย</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>ถ้ามี edge features (chapter→character)</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>codex แสดง chapter/note ด้วย (ไม่ได้ซ่อนเหมือน World Graph)</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>ต่ำ</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr"/>
+      <c r="G11" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(factions): overhaul faction system + timeline conflicts + proofread tags
Faction system:
- schema: hierarchy (parentFactionId), status, alignment, goal, element,
  leaderId; new faction_relationships table (ally/enemy/subsidiary/...)
- new /factions page: status board + tree view, drag across status,
  drag-to-reparent (dnd-kit, cycle-guarded), inspector with inline edit,
  faction<->faction relationships; on-brand forge/steel styling
- server: faction-relationship CRUD + autoLinkFactions(name->id) for
  future Story Bible import
- assistant: CRUD_FORMAT.faction gains status/alignment/goal/element

Also from this session:
- plot board: inline timeline-conflicts panel (B1)
- rewrite: per-paragraph proofread tags
- test-cases.xlsx: new "Factions (ใหม่)" sheet (24 cases)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-cases.xlsx
+++ b/test-cases.xlsx
@@ -16,6 +16,7 @@
     <sheet name="Stylometry เจาะลึก" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Context Fabric P4" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Story Codex (B1)" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Factions (ใหม่)" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ผู้ช่วย AI (ใหม่)'!$A$1:$G$19</definedName>
@@ -91,7 +92,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -113,11 +114,25 @@
         <color rgb="00D0D0D0"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -145,6 +160,13 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -511,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -695,6 +717,774 @@
       <c r="B18" t="n">
         <v>10</v>
       </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Factions (ใหม่)</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>หัวข้อ</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>เงื่อนไข / ขั้นตอน</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>ผลที่คาดหวัง</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>ความสำคัญ</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>ผลทดสอบ</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>หมายเหตุ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>F-01</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>เปิดหน้า Factions</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>คลิกเมนู Factions (ไอคอนโล่) ในกลุ่ม 'สร้างโลก'</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>เข้าหน้า /factions ได้ เห็น status board 5 คอลัมน์ (ยังปฏิบัติการ/ร่วมกับรัฐ/ย้ายฝั่ง/ไม่สังกัด/สาบสูญ) หรือ empty state ถ้ายังไม่มีฝ่าย</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr"/>
+      <c r="G2" s="12" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>F-02</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>สร้างฝ่ายใหม่</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>กด 'เพิ่มฝ่าย' &gt; กรอกชื่อ 'กปธ.' เลือกสถานะ 'ร่วมกับรัฐ' จุดยืน 'สีเทา' &gt; กด สร้าง</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>การ์ด 'กปธ.' โผล่ในคอลัมน์ 'ร่วมกับรัฐ' มี badge 'สีเทา' toast 'สร้างฝ่ายแล้ว'</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr"/>
+      <c r="G3" s="12" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>F-03</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>สร้างโดยไม่ใส่ชื่อ</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>กด 'เพิ่มฝ่าย' &gt; เว้นชื่อว่าง &gt; กด สร้าง</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>ขึ้น error 'ใส่ชื่อฝ่ายก่อนนะครับ' ไม่มีการสร้าง</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr"/>
+      <c r="G4" s="12" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>F-04</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>แก้ไขฝ่าย</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>คลิกการ์ดฝ่าย &gt; แก้เป้าหมาย/สี &gt; กด บันทึก</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>การ์ดอัปเดตทันที (สี/เป้าหมาย) toast 'บันทึกแล้ว'</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr"/>
+      <c r="G5" s="12" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>F-05</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>เปลี่ยนสถานะแล้วย้ายคอลัมน์</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>แก้ฝ่ายให้สถานะ = 'สาบสูญ' &gt; บันทึก</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>การ์ดย้ายไปคอลัมน์ 'สาบสูญ/ยุบ'</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr"/>
+      <c r="G6" s="12" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>F-06</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>ลำดับชั้น (parent)</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>สร้าง 'แผนกสรรพาวุธ' &gt; ตั้ง 'สังกัดใต้ฝ่าย' = กปธ. &gt; บันทึก</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>การ์ดแสดง '↳ ใต้ กปธ.'</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr"/>
+      <c r="G7" s="12" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>F-07</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>กำหนดหัวหน้า</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>เลือกตัวละครใน dropdown 'หัวหน้า' &gt; บันทึก</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>การ์ดแสดงชื่อหัวหน้าพร้อมไอคอนมงกุฎ (ต้องมีตัวละครในโปรเจกต์ก่อน)</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr"/>
+      <c r="G8" s="12" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>F-08</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>faction relationship (เพิ่ม)</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>เปิดฝ่าย A &gt; ส่วนความสัมพันธ์ เลือกชนิด 'ศัตรู' + ฝ่าย B &gt; กด +</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>รายการ 'ศัตรู → B' โผล่ในลิสต์ toast 'เพิ่มความสัมพันธ์แล้ว'</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr"/>
+      <c r="G9" s="12" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>F-09</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>relationship แสดงสองทาง</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>เปิดฝ่าย B (ปลายทางของ F-08)</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>เห็นรายการ '← ศัตรู B' (ทิศทางเข้า)</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr"/>
+      <c r="G10" s="12" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>F-10</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>relationship กับตัวเอง</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>เลือกฝ่ายปลายทาง = ฝ่ายเดียวกับที่เปิดอยู่ &gt; กด +</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>error 'เลือกฝ่ายอื่นที่ไม่ใช่ตัวเอง' ไม่มีการสร้าง</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr"/>
+      <c r="G11" s="12" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>F-11</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>ลบ relationship</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>hover รายการความสัมพันธ์ &gt; กดกากบาท</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>รายการหายไป toast 'ลบความสัมพันธ์แล้ว'</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr"/>
+      <c r="G12" s="12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>F-12</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>ลบฝ่าย</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>เปิดฝ่าย &gt; กดถังขยะ &gt; ยืนยัน</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>ฝ่ายหายจาก board, ความสัมพันธ์ที่ผูกไว้หายด้วย, panel ปิด toast 'ลบแล้ว'</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr"/>
+      <c r="G13" s="12" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>F-13</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>สมาชิก (อ่านอย่างเดียว)</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>เปิดฝ่ายที่มีสมาชิก (assign จากหน้า Relationships มาก่อน)</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>ส่วน 'สมาชิก' แสดงรายชื่อ+บทบาท; ถ้าไม่มีขึ้นข้อความให้ไปเพิ่มที่หน้า Characters/Relationships</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F14" s="12" t="inlineStr"/>
+      <c r="G14" s="12" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>F-14</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>ผู้ช่วย AI สร้าง faction พร้อม field ใหม่</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>ในผู้ช่วยพิมพ์ 'สร้างฝ่ายชื่อ ตระกูลอัคนีศวร สถานะ disbanded จุดยืน gray' &gt; ยืนยันร่าง</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>สร้างฝ่ายลงคอลัมน์ 'สาบสูญ/ยุบ' พร้อม alignment 'สีเทา'</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr"/>
+      <c r="G15" s="12" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>F-15</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>ข้อมูลเดิมไม่พัง</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>เปิดหน้า Relationships เดิม สร้าง/ลบ faction แบบเดิม</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>ยังทำงานได้ปกติ (ไม่ regression จากการเพิ่มคอลัมน์)</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F16" s="12" t="inlineStr"/>
+      <c r="G16" s="12" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>F-16</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>สลับมุมมอง</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>กดปุ่ม 'ลำดับชั้น' ในแถบบน</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>สลับจาก status board เป็น tree view; กด 'สถานะ' กลับได้</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr"/>
+      <c r="G17" s="12" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>F-17</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>Tree แสดงลำดับชั้น</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>ในมุมมองลำดับชั้น เปิดฝ่ายที่มี parent</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>ฝ่ายลูกเยื้องอยู่ใต้ฝ่ายแม่ พร้อมปุ่ม chevron พับ/ขยาย</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="inlineStr"/>
+      <c r="G18" s="12" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>F-18</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>พับ/ขยาย tree</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>กด chevron หน้าฝ่ายแม่</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>ซ่อน/แสดงฝ่ายลูกได้</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>ต่ำ</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr"/>
+      <c r="G19" s="12" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>F-19</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>ลากย้ายข้ามสถานะ</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>ใน status board ลากการ์ดจากคอลัมน์หนึ่งไปอีกคอลัมน์</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>การ์ดย้ายคอลัมน์ทันที (optimistic) toast 'ย้ายไป ...'; refresh แล้วยังอยู่คอลัมน์ใหม่</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F20" s="12" t="inlineStr"/>
+      <c r="G20" s="12" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>F-20</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>ลาก re-parent ใน tree</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>ลากการ์ด A วางบนการ์ด B</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>A กลายเป็นลูกของ B (เยื้องเข้า) toast 'ย้ายไปใต้ B'</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F21" s="12" t="inlineStr"/>
+      <c r="G21" s="12" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>F-21</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>กัน cycle</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>ลากฝ่ายแม่วางบนฝ่ายลูกของตัวเอง</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>error 'ย้ายเข้าใต้ฝ่ายลูกของตัวเองไม่ได้' ไม่มีการเปลี่ยน</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr"/>
+      <c r="G22" s="12" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>F-22</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>ลากขึ้น root</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>ในมุมมอง tree ลากฝ่ายลูกไปวางพื้นที่ว่าง (ไม่ใช่การ์ด)</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>parent ถูกล้าง ฝ่ายเลื่อนขึ้นบนสุด toast 'ย้ายขึ้นบนสุด'</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F23" s="12" t="inlineStr"/>
+      <c r="G23" s="12" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>F-23</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>คลิกยังเปิด inspector ได้</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>คลิกการ์ด (ไม่ลาก)</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>เปิด panel แก้ไข ไม่สับสนกับการลาก (distance 6px)</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="F24" s="12" t="inlineStr"/>
+      <c r="G24" s="12" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>F-24</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>autoLinkFactions (server)</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>เรียก autoLinkFactions(novelId, [{name:'แผนกสรรพาวุธ', parentName:'กปธ.'}]) เมื่อมีทั้งสองฝ่าย</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>คืน {linked:1}; แผนกสรรพาวุธมี parent = กปธ.; ชื่อซ้ำ/ไม่เจอ อยู่ใน unresolved</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr"/>
+      <c r="G25" s="12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(plot): idea-level participants + thread ribbon + POV + therefore/but causal chain
- SceneParticipantsPanel reworked to idea-in-scene scope (reuses scene_element_details, adds role column)
- ThreadRibbon (L3): per-thread lanes across chapters — beat dots, open-thread tails, stale-gap warnings
- POV per scene (P1): povCharacterId + dropdown in dramatic panel + eye badge on event cards
- Causal chain (P2): causeEventId/causeKind/causeNote — therefore/but buttons, 'and then' weak-link badge on board
- test-cases.xlsx: 3 new sheets

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-cases.xlsx
+++ b/test-cases.xlsx
@@ -17,6 +17,10 @@
     <sheet name="Context Fabric P4" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Story Codex (B1)" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Factions (ใหม่)" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="ผู้เข้าร่วมไอเดีย (ใหม่)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="เลนปม Ribbon (ใหม่)" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="POV ต่อฉาก (ใหม่)" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="ห่วงโซ่เหตุ-ผล (ใหม่)" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ผู้ช่วย AI (ใหม่)'!$A$1:$G$19</definedName>
@@ -1491,6 +1495,1299 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>หัวข้อ</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>เงื่อนไข / ขั้นตอน</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>ผลที่คาดหวัง</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>ความสำคัญ</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>ผลทดสอบ</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>หมายเหตุ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>IP-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ปุ่มผู้เข้าร่วมบน idea card</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>เปิดฉากใน Plot Board &gt; ดู idea card ที่มี children</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ท้ายการ์ดมีปุ่ม 'ผู้เข้าร่วม (n)' แทนปุ่ม 'เพิ่ม Dummy' เดิม โดย n = จำนวนตัวละคร/ฝ่าย (ไม่นับ location/sticky note)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>IP-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>เพิ่มตัวละครจริง</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>กดปุ่มผู้เข้าร่วม &gt; ประเภท 'ตัวละครจริง' &gt; เลือกตัวละคร + บทบาท 'ฝ่ายตรงข้าม' &gt; กรอก action/outcome &gt; กด เพิ่มเข้าไอเดีย</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ตัวละครโผล่ทั้งใน list ของ panel (พร้อม role badge สีแดง) และในหมวด Characters ของการ์ด, toast 'เพิ่มผู้เข้าร่วมแล้ว'</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>IP-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>เพิ่มกลุ่มฝ่ายจริง</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ประเภท 'กลุ่มฝ่ายจริง' &gt; เลือก faction &gt; เพิ่ม</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>faction โผล่ในหมวด Factions ของการ์ด (ไอคอนโล่เขียว)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>IP-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>เพิ่ม Dummy</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ประเภท 'ตัวละครชั่วคราว (Dummy)' &gt; กรอกชื่อ 'ทหารยาม' &gt; เพิ่ม</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>แสดง 'ทหารยาม (Dummy)' กรอบเส้นประ ทั้งใน panel และในการ์ด</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>IP-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Validation ค่าว่าง</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>กดเพิ่มโดยไม่เลือกตัวละคร / เลือก Dummy แต่ไม่กรอกชื่อ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>toast error 'กรุณาเลือกตัวละครหรือกลุ่มฝ่าย' / 'กรุณากรอกชื่อ Dummy' ไม่มีการเพิ่ม</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>IP-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>กันเพิ่มซ้ำ</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>เพิ่มตัวละครคนเดิมซ้ำในไอเดียเดียวกัน</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>toast 'มีผู้เข้าร่วมนี้ในไอเดียแล้ว' ไม่มีรายการซ้ำ</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>IP-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>แก้ไข inline</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ใน panel คลิกบรรทัด action/outcome ของผู้เข้าร่วม &gt; แก้ action, outcome, เปลี่ยนบทบาท &gt; บันทึก</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ค่าอัปเดตทันที role badge เปลี่ยนสีตามบทบาทใหม่, toast 'อัปเดตข้อมูลผู้เข้าร่วมแล้ว'</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>IP-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ลบผู้เข้าร่วม</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>hover รายการใน panel &gt; กดไอคอนถังขยะ</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>หายจากทั้ง panel และการ์ด, toast 'ลบผู้เข้าร่วมแล้ว'</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>IP-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ข้อมูลคงอยู่หลัง refresh</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>เพิ่มผู้เข้าร่วม + action &gt; กด Save canvas &gt; refresh หน้า</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ผู้เข้าร่วม role action/outcome แสดงครบเหมือนก่อน refresh</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>IP-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ใช้ record เดียวกับ dialog ดินสอ</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>เพิ่มผ่าน panel &gt; กดดินสอที่ child ในการ์ด &gt; กรอก how/goal &gt; บันทึก &gt; กลับมาแก้ role ใน panel</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>how/goal ที่กรอกใน dialog ไม่หายหลังแก้ role ผ่าน panel (เก็บใน record เดียวกัน)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>IP-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>สโคปแยกต่อไอเดีย</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>สร้าง 2 idea cards ในฉากเดียว เพิ่มตัวละครคนเดียวกันทั้ง 2 การ์ด ให้ role ต่างกัน</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>แต่ละการ์ดเก็บ role/action ของตัวเอง ไม่ทับกัน</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>IP-12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Migration คอลัมน์ role</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>รัน npm run db:push ก่อนทดสอบทั้งหมด</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>push สำเร็จ มีคอลัมน์ role ใน scene_element_details / ถ้าไม่รัน การบันทึกจะ error</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>หัวข้อ</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>เงื่อนไข / ขั้นตอน</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>ผลที่คาดหวัง</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>ความสำคัญ</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>ผลทดสอบ</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>หมายเหตุ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>RB-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>เปิดเลนปม</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>หน้า Plot Board &gt; ปุ่ม 'มุมมอง' &gt; toggle 'เลนปม'</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>แสดงแถบเลนปมใต้ arc strip/เส้น tension, ตัวเลข badge บนปุ่มมุมมองเพิ่มขึ้น 1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>RB-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Empty state</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>เปิดเลนปมทั้งที่ยังไม่มีปมผูกกับฉากใดเลย</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ข้อความ 'เลนปม — ผูกปมเข้ากับฉากผ่านสมุดปมเพื่อเริ่มวาดเลน'</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>RB-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>เส้นเลนต่อปม</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>สร้างปม 1 อัน ผูก beat 'หว่าน' ที่ฉากบท 2 และ 'เฉลย' ที่ฉากบท 5</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>เลนของปมมีเส้นสีของปมพาดจากกลางคอลัมน์บท 2 ถึงบท 5 จุดบท 2 สีเหลือง (หว่าน) จุดบท 5 สีเขียวใหญ่กว่า (เฉลย)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>RB-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>จุด 'ย้ำ'</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>เพิ่ม beat 'ย้ำ' ที่บท 3 ของปมเดิม</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>จุดสีน้ำเงินโผล่ที่บท 3 บนเลนเดียวกัน</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>RB-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ปมค้าง (หางเส้นประ)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ปมสถานะ 'หว่านแล้ว/กำลังสาน' beat สุดท้ายอยู่บทกลางเรื่อง</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>เส้นประจางลากจากบท beat สุดท้ายถึงบทสุดท้าย + ตัวหนังสือแดง 'ค้าง' ท้ายเลน + จุดแดงหลังชื่อปม</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>RB-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ปมเฉลยแล้วไม่ค้าง</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ปมสถานะ 'เฉลยแล้ว'</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>เส้นจบที่บทเฉลย ไม่มีเส้นประ ไม่มีคำว่า 'ค้าง'</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>RB-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ช่วงเงียบเกิน 8 บท</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ปมมี beat บท 1 แล้ว beat ถัดไปบท 10 ขึ้นไป (ห่างเกิน 8 บท)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ช่วงว่างระหว่างสองจุดทาบด้วยแถบแดงจาง (เตือนผู้อ่านลืม)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>RB-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>เรียง major ก่อน</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>มีปม major และ minor</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>เลนของปม major อยู่บนสุด เส้นหนากว่า ชื่อตัวหนา</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>RB-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ชื่อปม sticky</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>scroll กระดานไปทางขวาไกลๆ</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ป้ายชื่อปมยังติดขอบซ้ายจอ อ่านได้ตลอด</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RB-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>หลาย beat บทเดียว</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ผูก 2 beats ของปมเดียวกันกับ 2 ฉากในบทเดียวกัน</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>จุดเดียวพร้อมตัวเลข ×2 เหนือจุด สี = role สูงสุด (เฉลย &gt; ย้ำ &gt; หว่าน)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ต่ำ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>RB-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>แนวตรงกับคอลัมน์</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>เปิดเลนปม + เส้น tension พร้อมกัน</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>จุดบนเลนและจุดบนเส้น tension อยู่กึ่งกลางคอลัมน์บทเดียวกัน (แนว x ตรงกัน)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>หัวข้อ</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>เงื่อนไข / ขั้นตอน</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>ผลที่คาดหวัง</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>ความสำคัญ</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>ผลทดสอบ</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>หมายเหตุ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PV-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Migration</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>รัน npm run db:push ก่อนทดสอบ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>push สำเร็จ มีคอลัมน์ pov_character_id ใน timeline_events</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PV-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>dropdown POV ใน panel</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>เข้าฉากใน Plot Board &gt; กด 'โครงฉากดราม่า'</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>มี dropdown 'มุมมอง (POV) — เล่าผ่านสายตาใคร' อยู่บนสุด ค่าเริ่มต้น '— ยังไม่กำหนด —' มีรายชื่อตัวละครทั้งหมด</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PV-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>บันทึก POV</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>เลือกตัวละคร &gt; กด บันทึกโครงฉาก &gt; ปิด-เปิด popover ใหม่</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ค่า POV ที่เลือกยังอยู่, toast 'บันทึกโครงฉากแล้ว'</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PV-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>badge บนการ์ดฉาก</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>กลับไปหน้ากระดานพล็อต ดูการ์ดฉากที่ตั้ง POV ไว้</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>มุมล่างซ้ายการ์ดมีไอคอนตา + ชื่อตัวละคร (สีม่วง) หน้า event type</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PV-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ล้าง POV</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>เปิด panel &gt; เปลี่ยนเป็น '— ยังไม่กำหนด —' &gt; บันทึก</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>badge ตาหายจากการ์ด, DB เก็บ null</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PV-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ลบตัวละครที่เป็น POV</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ลบตัวละครที่ถูกตั้งเป็น POV ของฉากใดฉากหนึ่ง</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ฉากไม่พัง — pov_character_id เป็น null (on delete set null), badge หาย</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PV-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>POV กับปุ่ม hasData</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ฉากที่ตั้งแค่ POV (ไม่มี goal/conflict)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ปุ่ม 'โครงฉากดราม่า' เปลี่ยนเป็นสี amber (นับว่ามีข้อมูลแล้ว)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ต่ำ</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>หัวข้อ</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>เงื่อนไข / ขั้นตอน</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>ผลที่คาดหวัง</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>ความสำคัญ</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>ผลทดสอบ</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>หมายเหตุ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CC-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Migration</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>รัน npm run db:push</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>มีคอลัมน์ cause_event_id / cause_kind / cause_note ใน timeline_events</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CC-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ตัวเลือกใน panel</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>เข้าฉาก &gt; โครงฉากดราม่า</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>มีส่วน 'ฉากนี้ต่อจากเรื่องก่อนหน้าแบบไหน' ปุ่ม 3 ตัว: ดังนั้น (เขียว) / แต่ว่า (แดง) / แล้วก็… (เทา ค่าเริ่มต้น)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CC-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>เลือก 'ดังนั้น' + ฉากต้นเหตุ</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>กด 'ดังนั้น' &gt; โผล่ dropdown ฉากต้นเหตุ + ช่อง note &gt; เลือกฉากอื่น กรอก note &gt; บันทึก</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>บันทึกสำเร็จ เปิด panel ใหม่ค่ายังอยู่ครบ</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CC-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>เลือก 'แต่ว่า' ไม่ระบุฉาก</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>กด 'แต่ว่า' &gt; ปล่อย dropdown เป็น '— ฉากก่อนหน้า / ไม่ระบุ —' &gt; บันทึก</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>บันทึกได้ cause_kind='but' cause_event_id=null</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CC-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>สลับกลับเป็น 'แล้วก็'</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ฉากที่ตั้ง 'ดังนั้น' ไว้ &gt; กด 'แล้วก็…' &gt; บันทึก</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ทั้ง kind/event/note ถูกล้างเป็น null</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CC-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>badge บนการ์ด</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ดูกระดานพล็อต</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ฉากที่ตั้ง 'ดังนั้น' มีคำเขียว, 'แต่ว่า' มีคำแดง, ฉากที่ยังไม่ตั้ง (ยกเว้นฉากแรกสุดของเรื่อง) มี 'แล้วก็…' สีเทาขีดเส้นประ = จุดอ่อนพล็อตมองเห็นได้ทั้งบอร์ด</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CC-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ฉากแรกไม่โดนเตือน</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ดูฉากแรกสุดของเรื่อง (คอลัมน์ S ใบแรก)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ไม่มี badge 'แล้วก็…'</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CC-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>tooltip</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>hover badge ดังนั้น/แต่ว่า ที่มี note</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>แสดง cause_note ที่กรอกไว้</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ต่ำ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CC-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ลบฉากต้นเหตุ</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ลบฉากที่ถูกอ้างเป็น cause ของฉากอื่น</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ฉากปลายทางไม่พัง cause_event_id เป็น null แต่ kind/note ยังอยู่</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat(plot): typed canvas links + auto-arrange + real-world chronology (P3)
- Canvas links now carry kind (related/leads_to/conflicts/simultaneous) + label; click a line to edit or delete (backward-compatible with legacy string links)
- Children copy moved from link-creation to setting kind 'leads_to'
- Auto-arrange button: ideas laid out left-to-right by leads_to chain, undo via toast
- storyTimeIndex column + 'เวลาในเรื่อง' field in dramatic panel
- ChronoTimelineSheet: drag-order scenes by in-world time, flashback rows highlighted with badge count
- test-cases.xlsx: 2 new sheets

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-cases.xlsx
+++ b/test-cases.xlsx
@@ -21,6 +21,8 @@
     <sheet name="เลนปม Ribbon (ใหม่)" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="POV ต่อฉาก (ใหม่)" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="ห่วงโซ่เหตุ-ผล (ใหม่)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="เส้น Link มีชนิด (ใหม่)" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="จัดระเบียบ+เส้นเวลา (ใหม่)" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ผู้ช่วย AI (ใหม่)'!$A$1:$G$19</definedName>
@@ -2788,6 +2790,666 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>หัวข้อ</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>เงื่อนไข / ขั้นตอน</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>ผลที่คาดหวัง</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>ความสำคัญ</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>ผลทดสอบ</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>หมายเหตุ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>LK-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>เส้นเก่ายังแสดง</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>เปิดฉากที่มีเส้น link เดิม (สร้างก่อนอัปเดต)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>เส้นด้ายแดงเดิมแสดงปกติ = ชนิด 'เกี่ยวข้อง'</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>LK-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>สร้างเส้นใหม่</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>กดปุ่ม link บนการ์ด &gt; คลิกการ์ดปลายทาง</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ได้เส้นแดง 'เกี่ยวข้อง' และ **ไม่มี** การ copy ตัวละครไปปลายทางอีกแล้ว (เปลี่ยนพฤติกรรมจากเดิม)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>LK-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>คลิกเส้นเพื่อแก้</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>คลิกที่เส้น link บน canvas</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>เปิด dialog 'เส้นเชื่อม A → B' มีปุ่มชนิด 4 แบบ + ช่อง label + ปุ่มลบเส้น</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LK-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ชนิด 'นำไปสู่'</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>เปลี่ยนชนิดเป็น 'นำไปสู่' &gt; บันทึก</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>เส้นเปลี่ยนเป็นสีเขียว + หัวลูกศรชี้ปลายทาง และตัวละครใน card ต้นทางถูก copy ไปปลายทาง (toast แจ้ง) ตัวซ้ำไม่ถูก copy ซ้ำ</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LK-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ชนิด 'ขัดแย้งกับ'</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>เปลี่ยนเป็น 'ขัดแย้งกับ'</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>เส้นแดงเส้นประ ไม่ copy อะไร</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LK-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ชนิด 'เกิดพร้อมกัน'</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>เปลี่ยนเป็น 'เกิดพร้อมกัน'</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>เส้นน้ำเงินทึบ</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>LK-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>label บนเส้น</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>พิมพ์ label 'เพราะโดนหักหลัง' &gt; บันทึก</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ป้ายข้อความลอยกลางเส้น สีตามชนิดเส้น</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LK-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ลบเส้น</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>คลิกเส้น &gt; ปุ่ม 'ลบเส้น'</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>เส้นหาย toast 'ลบเส้นเชื่อมแล้ว'</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>LK-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>persist</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ตั้งชนิด/label &gt; กด Save canvas &gt; refresh</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ชนิด สี ลูกศร label แสดงเหมือนเดิมทุกเส้น</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>หัวข้อ</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>เงื่อนไข / ขั้นตอน</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>ผลที่คาดหวัง</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>ความสำคัญ</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>ผลทดสอบ</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>หมายเหตุ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AR-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ปุ่มจัดระเบียบ</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>canvas มี idea หลายใบ เชื่อม 'นำไปสู่' เป็น chain &gt; กดปุ่ม grid สีอำพันใน toolbar</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>idea เรียงซ้าย→ขวาตามลำดับ chain (ต้นเหตุซ้ายสุด), idea ไม่อยู่ใน chain อยู่คอลัมน์แรก, ของอื่นจัด grid ด้านล่าง, pan รีเซ็ต</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AR-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ย้อนกลับ</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>หลังกดจัดระเบียบ &gt; กด 'ย้อนกลับ' บน toast</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ทุก item กลับตำแหน่งเดิมก่อนจัด</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AR-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>chain วน</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>A นำไปสู่ B, B นำไปสู่ A &gt; กดจัดระเบียบ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ไม่ค้าง/ไม่ crash (กันวงจรแล้ว)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CT-01</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Migration</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>รัน npm run db:push</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>มีคอลัมน์ story_time_index ใน timeline_events</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CT-02</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ช่องเวลาในเรื่อง</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>เปิดโครงฉากดราม่า</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>มีช่อง 'เวลาในเรื่อง' กรอก text อิสระ บันทึกแล้วค่าคงอยู่</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CT-03</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>เปิด sheet เส้นเวลาจริง</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>กดปุ่ม 'เส้นเวลาจริง' บน toolbar กระดานพล็อต</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>side sheet เปิดจากขวา มีลิสต์ 'ยังไม่จัดลำดับ' ครบทุกฉาก (ยังไม่มีใครถูกจัด)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CT-04</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>เพิ่มเข้าเส้นเวลา</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>กด '+ เข้าเส้นเวลา' ทีละฉาก</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ฉากย้ายขึ้นลิสต์บน เรียงต่อท้าย มีเลข chrono กำกับ</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CT-05</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ลากเรียง</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ลากฉากในลิสต์บนสลับลำดับ</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ลำดับเปลี่ยน บันทึกอัตโนมัติ refresh แล้วคงอยู่</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CT-06</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ตรวจ flashback</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>จัดให้ฉากที่ 'เล่าทีหลัง' อยู่ก่อนตามเวลาจริง (เลขลำดับเล่าในลิสต์ไม่เรียง)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>แถวที่เล่าสลับ = พื้นอำพัน + ไอคอนนาฬิกา, ปุ่ม 'เส้นเวลาจริง' บน toolbar ขึ้น badge จำนวน flashback</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CT-07</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>เอาออกจากเส้นเวลา</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>hover แถว &gt; กด ✕</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ฉากกลับไปอยู่ 'ยังไม่จัดลำดับ' (storyTimeIndex = null)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>กลาง</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CT-08</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>kanban ไม่กระทบ</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ทำ CT-04..07 แล้วดูกระดานหลัก</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>คอลัมน์บท ลำดับการ์ด ไม่เปลี่ยนใดๆ</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>